<commit_message>
Update servo configurator, project manager, and calculator UI
- servo-app.js: refactor axis/motor logic and calculation flow
- configurator.html: UI tweaks and field updates
- project.html: improved layout and project management views
- titan-project-calculator.html: expanded calculator sections
- serve.py: streamlined static server setup
- titan_servo_input_template.xlsx: updated input template fields

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/titan_servo_input_template.xlsx
+++ b/titan_servo_input_template.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="4">
+  <fonts count="5">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -37,8 +37,11 @@
       <b val="1"/>
       <sz val="11"/>
     </font>
+    <font>
+      <b val="1"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="8">
     <fill>
       <patternFill/>
     </fill>
@@ -57,6 +60,26 @@
         <bgColor rgb="00FFFFE0"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFFFE0"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E2EFDA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="0092D050"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00ADD8E6"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -70,11 +93,26 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -440,12 +478,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C89"/>
+  <dimension ref="A1:C101"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="60" customWidth="1" min="1" max="1"/>
-    <col width="20" customWidth="1" min="2" max="2"/>
-    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="25" customWidth="1" min="2" max="2"/>
+    <col width="35" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -455,6 +493,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
@@ -473,7 +512,6 @@
           <t>OP90</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
@@ -486,13 +524,8 @@
           <t>App-1</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr"/>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr"/>
-      <c r="B6" t="inlineStr"/>
-      <c r="C6" t="inlineStr"/>
-    </row>
+    </row>
+    <row r="6"/>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
@@ -553,11 +586,7 @@
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" t="inlineStr"/>
-      <c r="B11" t="inlineStr"/>
-      <c r="C11" t="inlineStr"/>
-    </row>
+    <row r="11"/>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
@@ -603,11 +632,7 @@
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" t="inlineStr"/>
-      <c r="B15" t="inlineStr"/>
-      <c r="C15" t="inlineStr"/>
-    </row>
+    <row r="15"/>
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
         <is>
@@ -654,515 +679,509 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="3" t="inlineStr">
-        <is>
-          <t>Moving mass</t>
-        </is>
-      </c>
-      <c r="B19" t="n">
-        <v>1.6</v>
-      </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>kg</t>
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>External force direction</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="inlineStr">
+        <is>
+          <t>opposing movement</t>
+        </is>
+      </c>
+      <c r="C19" s="6" t="inlineStr">
+        <is>
+          <t>Options: opposing movement / aiding movement</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
         <is>
+          <t>Moving mass</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="inlineStr">
+        <is>
           <t>Tilt angle of the setup</t>
         </is>
       </c>
-      <c r="B20" t="n">
+      <c r="B21" t="n">
         <v>45</v>
       </c>
-      <c r="C20" t="inlineStr">
+      <c r="C21" t="inlineStr">
         <is>
           <t>deg</t>
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" t="inlineStr"/>
-      <c r="B21" t="inlineStr"/>
-      <c r="C21" t="inlineStr"/>
-    </row>
     <row r="22">
-      <c r="A22" s="3" t="inlineStr">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>Payload movement direction</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="inlineStr">
+        <is>
+          <t>against gravity</t>
+        </is>
+      </c>
+      <c r="C22" s="6" t="inlineStr">
+        <is>
+          <t>Options: against gravity / with gravity</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>Friction coefficient of linear guide (μ)</t>
+        </is>
+      </c>
+      <c r="B23" s="7" t="n">
+        <v>0.005</v>
+      </c>
+      <c r="C23" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="24"/>
+    <row r="25">
+      <c r="A25" s="3" t="inlineStr">
         <is>
           <t>Acceleration %</t>
         </is>
       </c>
-      <c r="B22" t="n">
+      <c r="B25" t="n">
         <v>25</v>
       </c>
-      <c r="C22" t="inlineStr">
+      <c r="C25" t="inlineStr">
         <is>
           <t>%</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="3" t="inlineStr">
-        <is>
-          <t>Safety factor %</t>
-        </is>
-      </c>
-      <c r="B23" t="n">
-        <v>20</v>
-      </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>%</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="3" t="inlineStr">
-        <is>
-          <t>Movement accuracy required (+/-)</t>
-        </is>
-      </c>
-      <c r="B24" t="n">
-        <v>10</v>
-      </c>
-      <c r="C24" t="inlineStr">
-        <is>
-          <t>micron</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="2" t="inlineStr">
-        <is>
-          <t>BALL SCREW DETAILS</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="3" t="inlineStr">
         <is>
-          <t>Selected Ball screw model</t>
-        </is>
-      </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>Festo - ESBF-BS-40-100-5P / 8022585</t>
-        </is>
-      </c>
-      <c r="C26" t="inlineStr"/>
+          <t>Safety factor %</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>20</v>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="3" t="inlineStr">
         <is>
-          <t>Ball screw Friction Torque @ application speed + no load torque</t>
+          <t>Movement accuracy required (+/-)</t>
         </is>
       </c>
       <c r="B27" t="n">
-        <v>0.05</v>
+        <v>10</v>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Nm @ 150 mm/sec</t>
+          <t>micron</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="3" t="inlineStr">
-        <is>
-          <t>Ball screw pitch</t>
-        </is>
-      </c>
-      <c r="B28" t="n">
-        <v>2</v>
-      </c>
-      <c r="C28" t="inlineStr">
-        <is>
-          <t>mm</t>
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>BALL SCREW DETAILS</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="3" t="inlineStr">
         <is>
-          <t>Ball screw dia</t>
-        </is>
-      </c>
-      <c r="B29" t="n">
-        <v>6</v>
-      </c>
-      <c r="C29" t="inlineStr">
-        <is>
-          <t>mm</t>
+          <t>Selected Ball screw model</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Festo - ESBF-BS-40-100-5P / 8022585</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>Ballscrew preload nut friction coefficient (μ0)</t>
+        </is>
+      </c>
+      <c r="B30" s="7" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="C30" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="2" t="inlineStr">
-        <is>
-          <t>PARALLEL KIT DETAILS</t>
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>Ballscrew preload force F0</t>
+        </is>
+      </c>
+      <c r="B31" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="C31" s="6" t="inlineStr">
+        <is>
+          <t>N</t>
         </is>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="3" t="inlineStr">
-        <is>
-          <t>Selected Parallel Kit Model</t>
-        </is>
-      </c>
-      <c r="B32" t="inlineStr">
-        <is>
-          <t>Festo - EAMM-U-60-D40-55A-91 / 1210438</t>
-        </is>
-      </c>
-      <c r="C32" t="inlineStr"/>
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>Ballscrew bearing drag torque</t>
+        </is>
+      </c>
+      <c r="B32" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="C32" s="6" t="inlineStr">
+        <is>
+          <t>Nm</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="3" t="inlineStr">
         <is>
-          <t>Gear Ratio</t>
+          <t>Ball screw pitch</t>
         </is>
       </c>
       <c r="B33" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>ratio</t>
+          <t>mm</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="3" t="inlineStr">
         <is>
-          <t>No Load Driving Torque</t>
+          <t>Ball screw dia</t>
         </is>
       </c>
       <c r="B34" t="n">
-        <v>0.07000000000000001</v>
+        <v>6</v>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Nm</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="3" t="inlineStr">
-        <is>
-          <t>Mass Moment of Inertia</t>
-        </is>
-      </c>
-      <c r="B35" t="n">
-        <v>26.7</v>
-      </c>
-      <c r="C35" t="inlineStr">
-        <is>
-          <t>kg·mm²</t>
-        </is>
-      </c>
-    </row>
+          <t>mm</t>
+        </is>
+      </c>
+    </row>
+    <row r="35"/>
     <row r="36">
-      <c r="A36" s="3" t="inlineStr">
-        <is>
-          <t>Max. Transferable torque</t>
-        </is>
-      </c>
-      <c r="B36" t="n">
-        <v>3</v>
-      </c>
-      <c r="C36" t="inlineStr">
-        <is>
-          <t>Nm</t>
+      <c r="A36" s="8" t="inlineStr">
+        <is>
+          <t>COUNTERBALANCE DETAILS</t>
         </is>
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="3" t="inlineStr">
-        <is>
-          <t>Max. Rotational Speed</t>
-        </is>
-      </c>
-      <c r="B37" t="n">
-        <v>6000</v>
-      </c>
-      <c r="C37" t="inlineStr">
-        <is>
-          <t>rpm</t>
+      <c r="A37" s="4" t="inlineStr">
+        <is>
+          <t>Counterbalance present</t>
+        </is>
+      </c>
+      <c r="B37" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="C37" s="6" t="inlineStr">
+        <is>
+          <t>Options: yes / no</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="4" t="inlineStr">
+        <is>
+          <t>Counterbalance mass</t>
+        </is>
+      </c>
+      <c r="B38" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="C38" s="6" t="inlineStr">
+        <is>
+          <t>kg</t>
         </is>
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="2" t="inlineStr">
-        <is>
-          <t>GUIDE DETAILS</t>
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t>Counterbalance inclination angle</t>
+        </is>
+      </c>
+      <c r="B39" s="7" t="n">
+        <v>90</v>
+      </c>
+      <c r="C39" s="6" t="inlineStr">
+        <is>
+          <t>deg</t>
         </is>
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="3" t="inlineStr">
-        <is>
-          <t>Selected Guide Model</t>
-        </is>
-      </c>
-      <c r="B40" t="inlineStr">
-        <is>
-          <t>Festo - EAGF-V2-KF-40-100 / 2782939</t>
-        </is>
-      </c>
-      <c r="C40" t="inlineStr"/>
-    </row>
-    <row r="41">
-      <c r="A41" s="3" t="inlineStr">
-        <is>
-          <t>Displacement Force required</t>
-        </is>
-      </c>
-      <c r="B41" t="n">
-        <v>15</v>
-      </c>
-      <c r="C41" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" s="3" t="inlineStr">
-        <is>
-          <t>Moving Mass</t>
-        </is>
-      </c>
-      <c r="B42" t="n">
-        <v>1.6</v>
-      </c>
-      <c r="C42" t="inlineStr">
-        <is>
-          <t>kg</t>
-        </is>
-      </c>
-    </row>
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t>Counterbalance friction coefficient (μ_cb)</t>
+        </is>
+      </c>
+      <c r="B40" s="7" t="n">
+        <v>0.005</v>
+      </c>
+      <c r="C40" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="41"/>
+    <row r="42"/>
     <row r="43">
-      <c r="A43" s="3" t="inlineStr">
-        <is>
-          <t>Max Withstand Force</t>
-        </is>
-      </c>
-      <c r="B43" t="n">
-        <v>1000</v>
-      </c>
-      <c r="C43" t="inlineStr">
-        <is>
-          <t>N</t>
+      <c r="A43" s="2" t="inlineStr">
+        <is>
+          <t>PARALLEL KIT DETAILS</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="3" t="inlineStr">
         <is>
-          <t>Service Life for 100% loading</t>
-        </is>
-      </c>
-      <c r="B44" t="n">
-        <v>5000</v>
-      </c>
-      <c r="C44" t="inlineStr">
-        <is>
-          <t>km</t>
+          <t>Selected Parallel Kit Model</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Festo - EAMM-U-60-D40-55A-91 / 1210438</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="3" t="inlineStr">
+        <is>
+          <t>Gear Ratio</t>
+        </is>
+      </c>
+      <c r="B45" t="n">
+        <v>1</v>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>ratio</t>
         </is>
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="2" t="inlineStr">
-        <is>
-          <t>GEAR BOX DETAILS</t>
+      <c r="A46" s="3" t="inlineStr">
+        <is>
+          <t>No Load Driving Torque</t>
+        </is>
+      </c>
+      <c r="B46" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>Nm</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="3" t="inlineStr">
         <is>
-          <t>Selected Gear Box Model</t>
-        </is>
-      </c>
-      <c r="B47" t="inlineStr">
-        <is>
-          <t>Not required here</t>
-        </is>
-      </c>
-      <c r="C47" t="inlineStr"/>
+          <t>Mass Moment of Inertia</t>
+        </is>
+      </c>
+      <c r="B47" t="n">
+        <v>26.7</v>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>kg·mm²</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="3" t="inlineStr">
         <is>
-          <t>Selected Gear ratio</t>
+          <t>Max. Transferable torque</t>
         </is>
       </c>
       <c r="B48" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>ratio</t>
+          <t>Nm</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="3" t="inlineStr">
         <is>
-          <t>Gearbox - Inertia</t>
+          <t>Max. Rotational Speed</t>
         </is>
       </c>
       <c r="B49" t="n">
-        <v>0</v>
+        <v>6000</v>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>kg·m²</t>
-        </is>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" s="3" t="inlineStr">
-        <is>
-          <t>GB - Efficiency</t>
-        </is>
-      </c>
-      <c r="B50" t="n">
-        <v>97</v>
-      </c>
-      <c r="C50" t="inlineStr">
-        <is>
-          <t>%</t>
-        </is>
-      </c>
-    </row>
+          <t>rpm</t>
+        </is>
+      </c>
+    </row>
+    <row r="50"/>
     <row r="51">
-      <c r="A51" s="3" t="inlineStr">
-        <is>
-          <t>GB - No load running torque</t>
-        </is>
-      </c>
-      <c r="B51" t="n">
-        <v>0.01</v>
-      </c>
-      <c r="C51" t="inlineStr">
-        <is>
-          <t>Nm</t>
+      <c r="A51" s="2" t="inlineStr">
+        <is>
+          <t>GUIDE DETAILS</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="3" t="inlineStr">
         <is>
-          <t>GB - Backlash</t>
-        </is>
-      </c>
-      <c r="B52" t="n">
-        <v>7</v>
-      </c>
-      <c r="C52" t="inlineStr">
-        <is>
-          <t>arcmin</t>
+          <t>Selected Guide Model</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>Festo - EAGF-V2-KF-40-100 / 2782939</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="3" t="inlineStr">
+        <is>
+          <t>Displacement Force required</t>
+        </is>
+      </c>
+      <c r="B53" t="n">
+        <v>15</v>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>N</t>
         </is>
       </c>
     </row>
     <row r="54">
-      <c r="A54" s="2" t="inlineStr">
-        <is>
-          <t>SERVO MOTOR DETAILS</t>
+      <c r="A54" s="3" t="inlineStr">
+        <is>
+          <t>Moving Mass</t>
+        </is>
+      </c>
+      <c r="B54" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>kg</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="3" t="inlineStr">
         <is>
-          <t>Selected Motor model</t>
-        </is>
-      </c>
-      <c r="B55" t="inlineStr">
-        <is>
-          <t>SIEMENS 1FL6042-1AF61-0LG1</t>
-        </is>
-      </c>
-      <c r="C55" t="inlineStr"/>
+          <t>Max Withstand Force</t>
+        </is>
+      </c>
+      <c r="B55" t="n">
+        <v>1000</v>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="3" t="inlineStr">
         <is>
-          <t>Rated RPM of selected Motor</t>
+          <t>Service Life for 100% loading</t>
         </is>
       </c>
       <c r="B56" t="n">
-        <v>3000</v>
+        <v>5000</v>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>rpm</t>
-        </is>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" s="3" t="inlineStr">
-        <is>
-          <t>SM - Rated torque</t>
-        </is>
-      </c>
-      <c r="B57" t="n">
-        <v>0.16</v>
-      </c>
-      <c r="C57" t="inlineStr">
-        <is>
-          <t>Nm</t>
-        </is>
-      </c>
-    </row>
+          <t>km</t>
+        </is>
+      </c>
+    </row>
+    <row r="57"/>
     <row r="58">
-      <c r="A58" s="3" t="inlineStr">
-        <is>
-          <t>SM - Peak Torque</t>
-        </is>
-      </c>
-      <c r="B58" t="n">
-        <v>0.24</v>
-      </c>
-      <c r="C58" t="inlineStr">
-        <is>
-          <t>Nm</t>
+      <c r="A58" s="2" t="inlineStr">
+        <is>
+          <t>GEAR BOX DETAILS</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="3" t="inlineStr">
         <is>
-          <t>SM - Rotor inertia</t>
-        </is>
-      </c>
-      <c r="B59" t="n">
-        <v>0.00027</v>
-      </c>
-      <c r="C59" t="inlineStr">
-        <is>
-          <t>kg·m²</t>
+          <t>Selected Gear Box Model</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>Not required here</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="3" t="inlineStr">
         <is>
-          <t>SM - Permitted Inertia Ratio</t>
+          <t>Selected Gear ratio</t>
         </is>
       </c>
       <c r="B60" t="n">
-        <v>7</v>
-      </c>
-      <c r="C60" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>ratio</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="3" t="inlineStr">
         <is>
-          <t>SM - Mechanical brake capacity</t>
+          <t>Gearbox - Inertia</t>
         </is>
       </c>
       <c r="B61" t="n">
@@ -1170,160 +1189,153 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>Nm</t>
+          <t>kg·m²</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="3" t="inlineStr">
         <is>
-          <t>SM - Encoder resolution</t>
+          <t>GB - Efficiency</t>
         </is>
       </c>
       <c r="B62" t="n">
-        <v>1048576</v>
+        <v>97</v>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>ppr</t>
+          <t>%</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="3" t="inlineStr">
         <is>
-          <t>Maximum RPM of selected Motor</t>
+          <t>GB - No load running torque</t>
         </is>
       </c>
       <c r="B63" t="n">
-        <v>4000</v>
+        <v>0.01</v>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>rpm</t>
+          <t>Nm</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="3" t="inlineStr">
         <is>
-          <t>SM - Service life (bearing)</t>
+          <t>GB - Backlash</t>
         </is>
       </c>
       <c r="B64" t="n">
-        <v>30000</v>
+        <v>7</v>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>hr</t>
-        </is>
-      </c>
-    </row>
-    <row r="65">
-      <c r="A65" s="3" t="inlineStr">
-        <is>
-          <t>SM - Mechanical brake service life</t>
-        </is>
-      </c>
-      <c r="B65" t="n">
-        <v>0</v>
-      </c>
-      <c r="C65" t="inlineStr">
-        <is>
-          <t>times</t>
+          <t>arcmin</t>
+        </is>
+      </c>
+    </row>
+    <row r="65"/>
+    <row r="66">
+      <c r="A66" s="2" t="inlineStr">
+        <is>
+          <t>SERVO MOTOR DETAILS</t>
         </is>
       </c>
     </row>
     <row r="67">
-      <c r="A67" s="2" t="inlineStr">
-        <is>
-          <t>ADDITIONAL BALL SCREW DETAILS</t>
+      <c r="A67" s="3" t="inlineStr">
+        <is>
+          <t>Selected Motor model</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>SIEMENS 1FL6042-1AF61-0LG1</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="3" t="inlineStr">
         <is>
-          <t>Ball screw rod length</t>
+          <t>Rated RPM of selected Motor</t>
         </is>
       </c>
       <c r="B68" t="n">
-        <v>124</v>
+        <v>3000</v>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>mm</t>
+          <t>rpm</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="3" t="inlineStr">
         <is>
-          <t>Ball screw efficiency</t>
+          <t>SM - Rated torque</t>
         </is>
       </c>
       <c r="B69" t="n">
-        <v>98</v>
+        <v>0.16</v>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>%</t>
+          <t>Nm</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="3" t="inlineStr">
         <is>
-          <t>Ball screw - permitted axial force max @ specified rod length</t>
+          <t>SM - Peak Torque</t>
         </is>
       </c>
       <c r="B70" t="n">
-        <v>3000</v>
+        <v>0.24</v>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>N @ 124 mm</t>
+          <t>Nm</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="3" t="inlineStr">
         <is>
-          <t>Ball screw - permitted axial force max @ application feed speed</t>
+          <t>SM - Rotor inertia</t>
         </is>
       </c>
       <c r="B71" t="n">
-        <v>3000</v>
+        <v>0.00027</v>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>N @ 150 mm/sec</t>
+          <t>kg·m²</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="3" t="inlineStr">
         <is>
-          <t>Ball screw - permitted radial force max</t>
+          <t>SM - Permitted Inertia Ratio</t>
         </is>
       </c>
       <c r="B72" t="n">
-        <v>90</v>
-      </c>
-      <c r="C72" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
+        <v>7</v>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="3" t="inlineStr">
         <is>
-          <t>Ball screw - Permitted driving torque max</t>
+          <t>SM - Mechanical brake capacity</t>
         </is>
       </c>
       <c r="B73" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="C73" t="inlineStr">
         <is>
@@ -1334,153 +1346,154 @@
     <row r="74">
       <c r="A74" s="3" t="inlineStr">
         <is>
-          <t>Ball screw - Permitted velocity @ specified stroke length</t>
+          <t>SM - Encoder resolution</t>
         </is>
       </c>
       <c r="B74" t="n">
-        <v>400</v>
+        <v>1048576</v>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>mm/sec @ 100 mm</t>
+          <t>ppr</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="3" t="inlineStr">
         <is>
-          <t>Ball screw - Permitted acceleration max</t>
+          <t>Maximum RPM of selected Motor</t>
         </is>
       </c>
       <c r="B75" t="n">
-        <v>5</v>
+        <v>4000</v>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>m/sec²</t>
+          <t>rpm</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="3" t="inlineStr">
         <is>
-          <t>Ball screw - Repetition accuracy (+/-)</t>
+          <t>SM - Service life (bearing)</t>
         </is>
       </c>
       <c r="B76" t="n">
-        <v>10</v>
+        <v>30000</v>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>micron</t>
+          <t>hr</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="3" t="inlineStr">
         <is>
-          <t>Ball screw - Moment of inertia</t>
+          <t>SM - Mechanical brake service life</t>
         </is>
       </c>
       <c r="B77" t="n">
-        <v>1.1e-05</v>
+        <v>0</v>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>kg·m²</t>
-        </is>
-      </c>
-    </row>
-    <row r="78">
-      <c r="A78" s="3" t="inlineStr">
-        <is>
-          <t>Ball screw - Moving mass (excluding spindle)</t>
-        </is>
-      </c>
-      <c r="B78" t="n">
-        <v>0.7</v>
-      </c>
-      <c r="C78" t="inlineStr">
-        <is>
-          <t>kg</t>
-        </is>
-      </c>
-    </row>
+          <t>times</t>
+        </is>
+      </c>
+    </row>
+    <row r="78"/>
     <row r="79">
-      <c r="A79" s="3" t="inlineStr">
-        <is>
-          <t>Ball screw - Duty cycle</t>
-        </is>
-      </c>
-      <c r="B79" t="n">
-        <v>100</v>
-      </c>
-      <c r="C79" t="inlineStr">
-        <is>
-          <t>%</t>
+      <c r="A79" s="2" t="inlineStr">
+        <is>
+          <t>ADDITIONAL BALL SCREW DETAILS</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="3" t="inlineStr">
         <is>
-          <t>Ball screw service life @ application axial force</t>
+          <t>Ball screw rod length</t>
         </is>
       </c>
       <c r="B80" t="n">
-        <v>30000</v>
+        <v>124</v>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>km @ 200 N</t>
+          <t>mm</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="3" t="inlineStr">
+        <is>
+          <t>Ball screw efficiency</t>
+        </is>
+      </c>
+      <c r="B81" t="n">
+        <v>98</v>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>%</t>
         </is>
       </c>
     </row>
     <row r="82">
-      <c r="A82" s="2" t="inlineStr">
-        <is>
-          <t>ADDITIONAL GEAR BOX DETAILS</t>
+      <c r="A82" s="3" t="inlineStr">
+        <is>
+          <t>Ball screw - permitted axial force max @ specified rod length</t>
+        </is>
+      </c>
+      <c r="B82" t="n">
+        <v>3000</v>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>N @ 124 mm</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="3" t="inlineStr">
         <is>
-          <t>GB - Rated Input Speed</t>
+          <t>Ball screw - permitted axial force max @ application feed speed</t>
         </is>
       </c>
       <c r="B83" t="n">
-        <v>0</v>
+        <v>3000</v>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>rpm</t>
+          <t>N @ 150 mm/sec</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="3" t="inlineStr">
         <is>
-          <t>GB - Max Input Speed</t>
+          <t>Ball screw - permitted radial force max</t>
         </is>
       </c>
       <c r="B84" t="n">
-        <v>0</v>
+        <v>90</v>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>rpm</t>
+          <t>N</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="3" t="inlineStr">
         <is>
-          <t>GB - Rated Output Torque</t>
+          <t>Ball screw - Permitted driving torque max</t>
         </is>
       </c>
       <c r="B85" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="C85" t="inlineStr">
         <is>
@@ -1491,58 +1504,216 @@
     <row r="86">
       <c r="A86" s="3" t="inlineStr">
         <is>
-          <t>GB - Max Output Torque</t>
+          <t>Ball screw - Permitted velocity @ specified stroke length</t>
         </is>
       </c>
       <c r="B86" t="n">
-        <v>0</v>
+        <v>400</v>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>Nm</t>
+          <t>mm/sec @ 100 mm</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="3" t="inlineStr">
         <is>
-          <t>GB - Permitted Radial Force</t>
+          <t>Ball screw - Permitted acceleration max</t>
         </is>
       </c>
       <c r="B87" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>m/sec²</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="3" t="inlineStr">
         <is>
-          <t>GB - Permitted Axial Force</t>
+          <t>Ball screw - Repetition accuracy (+/-)</t>
         </is>
       </c>
       <c r="B88" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>micron</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" s="3" t="inlineStr">
         <is>
+          <t>Ball screw - Moment of inertia</t>
+        </is>
+      </c>
+      <c r="B89" t="n">
+        <v>1.1e-05</v>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>kg·m²</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="3" t="inlineStr">
+        <is>
+          <t>Ball screw - Moving mass (excluding spindle)</t>
+        </is>
+      </c>
+      <c r="B90" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="3" t="inlineStr">
+        <is>
+          <t>Ball screw - Duty cycle</t>
+        </is>
+      </c>
+      <c r="B91" t="n">
+        <v>100</v>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="3" t="inlineStr">
+        <is>
+          <t>Ball screw service life @ application axial force</t>
+        </is>
+      </c>
+      <c r="B92" t="n">
+        <v>30000</v>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>km @ 200 N</t>
+        </is>
+      </c>
+    </row>
+    <row r="93"/>
+    <row r="94">
+      <c r="A94" s="2" t="inlineStr">
+        <is>
+          <t>ADDITIONAL GEAR BOX DETAILS</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="3" t="inlineStr">
+        <is>
+          <t>GB - Rated Input Speed</t>
+        </is>
+      </c>
+      <c r="B95" t="n">
+        <v>0</v>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>rpm</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="3" t="inlineStr">
+        <is>
+          <t>GB - Max Input Speed</t>
+        </is>
+      </c>
+      <c r="B96" t="n">
+        <v>0</v>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>rpm</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="3" t="inlineStr">
+        <is>
+          <t>GB - Rated Output Torque</t>
+        </is>
+      </c>
+      <c r="B97" t="n">
+        <v>0</v>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>Nm</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="3" t="inlineStr">
+        <is>
+          <t>GB - Max Output Torque</t>
+        </is>
+      </c>
+      <c r="B98" t="n">
+        <v>0</v>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>Nm</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="3" t="inlineStr">
+        <is>
+          <t>GB - Permitted Radial Force</t>
+        </is>
+      </c>
+      <c r="B99" t="n">
+        <v>0</v>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" s="3" t="inlineStr">
+        <is>
+          <t>GB - Permitted Axial Force</t>
+        </is>
+      </c>
+      <c r="B100" t="n">
+        <v>0</v>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" s="3" t="inlineStr">
+        <is>
           <t>GB - Service life</t>
         </is>
       </c>
-      <c r="B89" t="n">
+      <c r="B101" t="n">
         <v>0</v>
       </c>
-      <c r="C89" t="inlineStr">
+      <c r="C101" t="inlineStr">
         <is>
           <t>hrs</t>
         </is>

</xml_diff>